<commit_message>
Added some columns in the data frames/excel sheets for the BSc students
</commit_message>
<xml_diff>
--- a/code/output/dat.type.token.sequential.explanation.xlsx
+++ b/code/output/dat.type.token.sequential.explanation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/endress/Experiments/Social learning through type and token frequency/sequential_BSc2022-23/code/output/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/endress/Experiments/Social learning through type and token frequency/sequential/code/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3755B2-6052-2C43-AAA9-DF5C902B9C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C0AC59-8617-0C4F-8D4E-5D2C55787FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1960" yWindow="-23500" windowWidth="38400" windowHeight="23500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="23500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Explanation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="83">
   <si>
     <t>filename</t>
   </si>
@@ -255,6 +255,33 @@
   </si>
   <si>
     <t>Gender</t>
+  </si>
+  <si>
+    <t>Machiavellianism.group</t>
+  </si>
+  <si>
+    <t>Narcissism.group</t>
+  </si>
+  <si>
+    <t>Psychopathy.group</t>
+  </si>
+  <si>
+    <t>mean.prevalence_raw</t>
+  </si>
+  <si>
+    <t>mean.third.party.acceptability_raw</t>
+  </si>
+  <si>
+    <t>mean.first.party.acceptablity_raw</t>
+  </si>
+  <si>
+    <t>Mean (across frequency conditions) for the prevalence rating</t>
+  </si>
+  <si>
+    <t>Mean (across frequency conditions) for the third party acceptability rating</t>
+  </si>
+  <si>
+    <t>Mean (across frequency conditions) for the first party acceptability rating</t>
   </si>
 </sst>
 </file>
@@ -362,7 +389,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -650,7 +677,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -658,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="44.1640625" bestFit="1" customWidth="1"/>
@@ -758,247 +785,256 @@
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="6"/>
-      <c r="B11" s="7"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" s="7"/>
+        <v>74</v>
+      </c>
+      <c r="B10" s="7" t="str">
+        <f>CONCATENATE(B6, "above or below median?")</f>
+        <v>Machiavellianism scoreabove or below median?</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="7" t="str">
+        <f>CONCATENATE(B7, "above or below median?")</f>
+        <v>Narcissism scoreabove or below median?</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="7" t="str">
+        <f>CONCATENATE(B8, "above or below median?")</f>
+        <v>Psychopathy scoreabove or below median?</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>51</v>
-      </c>
+      <c r="A13" s="6"/>
       <c r="B13" s="7"/>
     </row>
     <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="6"/>
+      <c r="B15" s="7"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B16" s="7"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="7"/>
+    </row>
+    <row r="18" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B18" s="7" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="6"/>
-      <c r="B17" s="7"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18" s="7"/>
     </row>
     <row r="19" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="6"/>
+      <c r="B21" s="7"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="7"/>
+    </row>
+    <row r="23" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B23" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="6" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="7"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="7"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="6"/>
-      <c r="B22" s="7"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>58</v>
-      </c>
+      <c r="B24" s="7"/>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="7"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="6"/>
+      <c r="B26" s="7"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="7"/>
+    </row>
+    <row r="28" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="7"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="6" t="s">
+      <c r="B29" s="7"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="7"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="6"/>
-      <c r="B27" s="7"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="8" t="s">
+      <c r="B30" s="7"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="6"/>
+      <c r="B31" s="7"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="7"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="8" t="s">
+      <c r="B32" s="7"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="7"/>
-    </row>
-    <row r="30" spans="1:2" ht="32" x14ac:dyDescent="0.2">
-      <c r="A30" s="6" t="s">
+      <c r="B33" s="7"/>
+    </row>
+    <row r="34" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B34" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="32" x14ac:dyDescent="0.2">
-      <c r="A31" s="6" t="s">
+    <row r="35" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B35" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="32" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
+    <row r="36" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B36" s="7" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="6"/>
-      <c r="B33" s="7"/>
-    </row>
-    <row r="34" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B35" s="7"/>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B36" s="7"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="6"/>
       <c r="B37" s="7"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="8" t="s">
+    <row r="38" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="7"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="7"/>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="6"/>
+      <c r="B41" s="7"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="7"/>
-    </row>
-    <row r="39" spans="1:2" ht="32" x14ac:dyDescent="0.2">
-      <c r="A39" s="6" t="s">
+      <c r="B42" s="7"/>
+    </row>
+    <row r="43" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B43" s="7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="32" x14ac:dyDescent="0.2">
-      <c r="A40" s="6" t="s">
+    <row r="44" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B44" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="32" x14ac:dyDescent="0.2">
-      <c r="A41" s="6" t="s">
+    <row r="45" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B45" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="6"/>
-      <c r="B42" s="7"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="6"/>
-      <c r="B43" s="7"/>
-    </row>
-    <row r="44" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="6"/>
+      <c r="B46" s="7"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="6"/>
+      <c r="B47" s="7"/>
+    </row>
+    <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A48" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B48" s="5" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" s="6"/>
-      <c r="B45" s="7"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B46" s="7"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B47" s="7"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B48" s="7"/>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="6"/>
@@ -1006,19 +1042,19 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B50" s="7"/>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B51" s="7"/>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B52" s="7"/>
     </row>
@@ -1028,19 +1064,19 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B54" s="7"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B55" s="7"/>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B56" s="7"/>
     </row>
@@ -1048,67 +1084,117 @@
       <c r="A57" s="6"/>
       <c r="B57" s="7"/>
     </row>
-    <row r="58" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A58" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B58" s="10"/>
-    </row>
-    <row r="59" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B59" s="10"/>
-    </row>
-    <row r="60" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A60" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B60" s="10"/>
-    </row>
-    <row r="61" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="9"/>
-      <c r="B61" s="10"/>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B58" s="7"/>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59" s="7"/>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60" s="7"/>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="6"/>
+      <c r="B61" s="7"/>
     </row>
     <row r="62" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B62" s="10"/>
     </row>
     <row r="63" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B63" s="10"/>
     </row>
     <row r="64" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B64" s="10"/>
+    </row>
+    <row r="65" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="9"/>
+      <c r="B65" s="10"/>
+    </row>
+    <row r="66" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A66" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B66" s="10"/>
+    </row>
+    <row r="67" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B67" s="10"/>
+    </row>
+    <row r="68" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B64" s="10"/>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A65" s="6"/>
-      <c r="B65" s="7"/>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A66" s="6" t="s">
+      <c r="B68" s="10"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="6"/>
+      <c r="B69" s="7"/>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B66" s="7"/>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A67" s="6" t="s">
+      <c r="B70" s="7"/>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B67" s="7"/>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A68" s="6" t="s">
+      <c r="B71" s="7"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B68" s="7"/>
+      <c r="B72" s="7"/>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="6"/>
+      <c r="B73" s="7"/>
+    </row>
+    <row r="74" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B74" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A75" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A76" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>82</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>